<commit_message>
Changed paths to dummy paths
</commit_message>
<xml_diff>
--- a/Source Code/data.xlsx
+++ b/Source Code/data.xlsx
@@ -442,10 +442,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -498,6 +498,25 @@
         <v>83.3</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>